<commit_message>
backup antes de alterações na impressão do EDC
</commit_message>
<xml_diff>
--- a/Docs/New/Versão Final Colinha ABIMAD 42 - EXPORTAÇÃO (Última Enviada EXW E FOB USD5).xlsx
+++ b/Docs/New/Versão Final Colinha ABIMAD 42 - EXPORTAÇÃO (Última Enviada EXW E FOB USD5).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="786" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="786" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Estofados KARAMS" sheetId="1" r:id="rId1"/>
@@ -341,11 +341,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="179" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="180" formatCode="0_ "/>
   </numFmts>
   <fonts count="45">
     <font>
@@ -1480,10 +1481,10 @@
     <xf numFmtId="3" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1909,7 +1910,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="251460" y="17489805"/>
+          <a:off x="251460" y="17423130"/>
           <a:ext cx="2327275" cy="1417955"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1991,7 +1992,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="342900" y="3430905"/>
+          <a:off x="342900" y="3364230"/>
           <a:ext cx="2327275" cy="1520825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2032,7 +2033,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="297180" y="5880735"/>
+          <a:off x="297180" y="5814060"/>
           <a:ext cx="2298700" cy="1513840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2073,7 +2074,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="274320" y="8635365"/>
+          <a:off x="274320" y="8568690"/>
           <a:ext cx="2327275" cy="1522730"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2114,7 +2115,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="281940" y="11056620"/>
+          <a:off x="281940" y="10989945"/>
           <a:ext cx="2298700" cy="1504315"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2155,7 +2156,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="365760" y="13616940"/>
+          <a:off x="365760" y="13550265"/>
           <a:ext cx="2298700" cy="1506220"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2191,7 +2192,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="575310" y="8043545"/>
+          <a:off x="575310" y="7976870"/>
           <a:ext cx="188595" cy="187960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2227,7 +2228,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="575310" y="10525760"/>
+          <a:off x="575310" y="10459085"/>
           <a:ext cx="188595" cy="187960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2263,7 +2264,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="639445" y="5296535"/>
+          <a:off x="639445" y="5229860"/>
           <a:ext cx="187960" cy="184785"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2299,7 +2300,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="575310" y="15732125"/>
+          <a:off x="575310" y="15665450"/>
           <a:ext cx="188595" cy="187960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2335,7 +2336,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="575310" y="19368770"/>
+          <a:off x="575310" y="19302095"/>
           <a:ext cx="188595" cy="189865"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2371,7 +2372,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="575310" y="12939395"/>
+          <a:off x="575310" y="12872720"/>
           <a:ext cx="188595" cy="187960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3198,7 +3199,8 @@
     <col min="6" max="6" width="11.1047619047619" style="1" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="16.552380952381" style="77" hidden="1" customWidth="1"/>
     <col min="8" max="9" width="11.1047619047619" style="1" customWidth="1"/>
-    <col min="10" max="11" width="12" style="77" customWidth="1"/>
+    <col min="10" max="10" width="12" style="77" customWidth="1"/>
+    <col min="11" max="11" width="18.2857142857143" style="77" customWidth="1"/>
     <col min="12" max="12" width="10.5714285714286" style="1" customWidth="1"/>
     <col min="13" max="13" width="12" style="1" customWidth="1"/>
     <col min="14" max="16384" width="8.88571428571429" style="1" customWidth="1"/>
@@ -3654,7 +3656,7 @@
       <c r="L12" s="43"/>
       <c r="M12" s="43"/>
     </row>
-    <row r="13" ht="21" spans="1:13">
+    <row r="13" spans="1:13">
       <c r="A13" s="74"/>
       <c r="B13" s="85" t="s">
         <v>17</v>
@@ -3681,20 +3683,20 @@
         <v>2455.99</v>
       </c>
       <c r="J13" s="95">
-        <f>I13+27.7044</f>
-        <v>2483.6944</v>
+        <f>SUM(J2:J9)</f>
+        <v>4604.7029</v>
       </c>
       <c r="K13" s="94">
-        <f>SUM(J2:J12)</f>
-        <v>4604.7029</v>
+        <f>SUM(K2:K9)</f>
+        <v>10462.65</v>
       </c>
       <c r="L13" s="96">
-        <f>SUM(K2:K12)</f>
-        <v>10462.65</v>
+        <f>SUM(L2:L12)</f>
+        <v>2092.53</v>
       </c>
       <c r="M13" s="97">
-        <f>L13+27.7044</f>
-        <v>10490.3544</v>
+        <f>SUM(M2:M12)</f>
+        <v>4241.2429</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -4044,16 +4046,16 @@
         <v>4395.4619</v>
       </c>
       <c r="K25" s="94">
-        <f t="shared" ref="K25:M25" si="4">J17+J18+J19+J20</f>
-        <v>4395.4619</v>
+        <f>SUM(K17:K21)</f>
+        <v>13016.05</v>
       </c>
       <c r="L25" s="109">
-        <f t="shared" si="4"/>
-        <v>13016.05</v>
+        <f>SUM(L17:L23)</f>
+        <v>2603.21</v>
       </c>
       <c r="M25" s="109">
-        <f t="shared" si="4"/>
-        <v>2603.21</v>
+        <f>SUM(M17:M24)</f>
+        <v>4344.6319</v>
       </c>
     </row>
     <row r="26" ht="14.4" customHeight="1" spans="1:13">
@@ -4397,16 +4399,16 @@
         <v>4802.9627</v>
       </c>
       <c r="K40" s="94">
-        <f t="shared" ref="K40:M40" si="5">SUM(J29:J39)</f>
-        <v>4802.9627</v>
+        <f>SUM(K29:K35)</f>
+        <v>9351.7</v>
       </c>
       <c r="L40" s="109">
-        <f t="shared" si="5"/>
-        <v>9351.7</v>
+        <f>SUM(L29:L39)</f>
+        <v>1870.34</v>
       </c>
       <c r="M40" s="109">
-        <f t="shared" si="5"/>
-        <v>1870.34</v>
+        <f>SUM(M29:M39)</f>
+        <v>4767.4327</v>
       </c>
     </row>
     <row r="41" ht="21" customHeight="1" spans="1:13">
@@ -4665,16 +4667,16 @@
         <v>2579.8719</v>
       </c>
       <c r="K52" s="94">
-        <f t="shared" ref="K52:M52" si="6">SUM(J43:J51)</f>
-        <v>2579.8719</v>
+        <f>SUM(K43:K50)</f>
+        <v>6207.55</v>
       </c>
       <c r="L52" s="109">
-        <f t="shared" si="6"/>
-        <v>6207.55</v>
+        <f>SUM(L43)</f>
+        <v>1241.51</v>
       </c>
       <c r="M52" s="109">
-        <f t="shared" si="6"/>
-        <v>1241.51</v>
+        <f>SUM(M43)</f>
+        <v>2448.6319</v>
       </c>
     </row>
     <row r="53" ht="15.6" customHeight="1" spans="1:13">
@@ -4965,16 +4967,16 @@
         <v>3364.5776</v>
       </c>
       <c r="K64" s="94">
-        <f t="shared" ref="K64:M64" si="7">SUM(J55:J63)</f>
-        <v>3364.5776</v>
+        <f>SUM(K55:K63)</f>
+        <v>10500.9</v>
       </c>
       <c r="L64" s="109">
-        <f t="shared" si="7"/>
-        <v>10500.9</v>
+        <f>SUM(L55:L63)</f>
+        <v>2100.18</v>
       </c>
       <c r="M64" s="109">
-        <f t="shared" si="7"/>
-        <v>2100.18</v>
+        <f>SUM(M55:M60)</f>
+        <v>3137.1176</v>
       </c>
     </row>
     <row r="65" ht="15.6" customHeight="1" spans="1:13">
@@ -5325,16 +5327,16 @@
         <v>4209.7528</v>
       </c>
       <c r="K78" s="94">
-        <f t="shared" ref="K78:M78" si="8">SUM(J67:J77)</f>
-        <v>4209.7528</v>
+        <f>SUM(K67:K71)</f>
+        <v>10676.85</v>
       </c>
       <c r="L78" s="109">
-        <f t="shared" si="8"/>
-        <v>10676.85</v>
+        <f>SUM(L67:L77)</f>
+        <v>2135.37</v>
       </c>
       <c r="M78" s="109">
-        <f t="shared" si="8"/>
-        <v>2135.37</v>
+        <f>SUM(M67:M77)</f>
+        <v>3857.0028</v>
       </c>
     </row>
     <row r="79" ht="14.4" customHeight="1" spans="1:13">
@@ -5772,16 +5774,16 @@
         <v>4299.4766</v>
       </c>
       <c r="K97" s="94">
-        <f t="shared" ref="K97:M97" si="9">SUM(J88:J96)</f>
-        <v>4299.4766</v>
+        <f>SUM(K88:K94)</f>
+        <v>12458.8</v>
       </c>
       <c r="L97" s="109">
-        <f t="shared" si="9"/>
-        <v>12458.8</v>
+        <f>SUM(L88:L94)</f>
+        <v>2491.76</v>
       </c>
       <c r="M97" s="109">
-        <f t="shared" si="9"/>
-        <v>2491.76</v>
+        <f>SUM(M88:M94)</f>
+        <v>3861.7266</v>
       </c>
     </row>
     <row r="98" ht="21" customHeight="1" spans="1:13">
@@ -7523,6 +7525,7 @@
     <col min="12" max="12" width="18.2857142857143" customWidth="1"/>
     <col min="13" max="13" width="16.3333333333333" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="18.2857142857143" customWidth="1"/>
     <col min="17" max="17" width="12" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>